<commit_message>
Put the horizon back to 2051; the pad manufactured scarcity
Solving to 2065 was adopted to push the terminal artefact outside the reported
window. Measured, it did not: exports gained one year (2038 -> 2039), because
14 extra years of held-flat demand against the same finite reserves drove the
Surat reserve dual from $0.00 to $14.42/GJ. The salvage half fell $8.64 ->
$6.14 as designed and the scarcity half more than replaced it.

That is a worse trade than it looks. The old rent was 100% terminal artefact on
a slack constraint; the new one is mostly a real dual, but on demand that was
invented by the padding rather than published. Swapping a terminal-value
artefact for a demand-padding artefact is not progress.

Reverting to the published-data horizon. The transport netting stays -- it is
right independently. The terminal value itself is the thing to fix.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q6cWJYUY3Yb9hp3dEuRK1M
</commit_message>
<xml_diff>
--- a/src/data/gary_parameters.xlsx
+++ b/src/data/gary_parameters.xlsx
@@ -495,7 +495,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2065</v>
+        <v>2051</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -504,7 +504,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Last SOLVED year. Well beyond horizon_report_end on purpose. The terminal salvage credit is de-discounted in get_scarcity_rents, so the Hotelling rent it implies grows at the discount rate and reaches the full salvage rate exactly at this year -- which means the last decade before it is contaminated by the horizon whatever the salvage price is. Solving to 2065 and reporting to 2050 puts that contaminated tail outside the window anyone reads. Series that end earlier (demand 2051, LNG prices 2051, GPG/industrial profiles 2045) hold their last published year across the padding; that is padding, not a forecast.</t>
+          <t>Last SOLVED year, one beyond horizon_report_end. Held at 2051 because that is where the published data ends (demand and ACIL Allen prices 2051, GPG/industrial profiles 2045). Padding further does NOT buy a cleaner answer: measured 2 Sep 2026, a 2065 pad put 14 extra years of held-flat demand against the same finite reserves and drove the Surat reserve dual from /bin/bash.00 to 4.42/GJ, manufacturing scarcity rather than removing an artefact. Fix the terminal value instead -- see TODO item 15.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify every ACIL Allen input against the public reports; fix attributions
Checked each ACIL-sourced value against the text of the two public AEMO-hosted
reports (Wholesale natural gas prices for AEMO, 14 Nov 2025; Natural gas price
forecasts for the Final 2023 IASR, 14 Jul 2023). All values match. Fixes:
- the cap-as-netback-ceiling quote is 2023 s2.6.1, not s4.1 (four places);
- LNG lever netbacks relabelled as GARY's derivation from ACIL's LNG price;
- Step 2 overlay cited to 2023 s2.4; Narrabri 2030 quoted from 2025 s4.1.1;
- README/inputs.md no longer credit the 2023 segment weights to the 2025 report.
docs/pricing.md gains a table of every ACIL input with report and section, and
lists the three inputs that are not ACIL's (netback deduction, OCGT premium,
foundation share).

Notes only: standard set re-solved to restamp provenance; results identical.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YDU1dyyyL9SkWKVZMbgk6k
</commit_message>
<xml_diff>
--- a/src/data/gary_parameters.xlsx
+++ b/src/data/gary_parameters.xlsx
@@ -1240,7 +1240,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Gas Market Code cap, ACIL Allen (14 Nov 2025) 2.3.1; applied as a ceiling on the LNG netback per ACIL Allen (14 Jul 2023) 4.1. Self-terminating: once the netback falls below it the ceiling stops binding.</t>
+          <t>Gas Market Code cap, ACIL Allen (14 Nov 2025) 2.3.1; applied as a ceiling on the LNG netback per ACIL Allen (14 Jul 2023) 2.6.1. Self-terminating: once the netback falls below it the ceiling stops binding.</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Weak global LNG demand: ACIL Allen's Accelerated Transition price path (netback $7.33/GJ in 2030, $3.94 by 2050)</t>
+          <t>Weak global LNG demand: ACIL Allen's Accelerated Transition LNG price path (14 Nov 2025, Table B.4). GARY's netback off it (less export_netback_deduction): $7.33/GJ in 2030, $3.94 by 2050</t>
         </is>
       </c>
     </row>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Strong global LNG demand: ACIL Allen's Slower Growth price path (netback $10.39/GJ in 2030, at the $12 Code cap from 2040)</t>
+          <t>Strong global LNG demand: ACIL Allen's Slower Growth LNG price path (14 Nov 2025, Table B.4). GARY's netback off it: $10.39/GJ in 2030, at the $12 Code cap from 2040</t>
         </is>
       </c>
     </row>

</xml_diff>